<commit_message>
multi branch students updates
</commit_message>
<xml_diff>
--- a/data/attendance/AMPHI_حموي_1_ثانوي.xlsx
+++ b/data/attendance/AMPHI_حموي_1_ثانوي.xlsx
@@ -20,7 +20,14 @@
     <comment ref="B5" authorId="0">
       <text>
         <r>
-          <t>student_id:a34881a6-554a-4624-9ae0-447737ddb951</t>
+          <t>student_id:5a0d8f4b-8d75-461a-ab32-f5e92ee50360</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0">
+      <text>
+        <r>
+          <t>student_id:54f4388c-8185-4058-9aa0-9f9ba272e60d</t>
         </r>
       </text>
     </comment>
@@ -29,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t>حموي 1 ثانوي  |  AMPHI  |  1AS  |  حموي عبد السلام</t>
   </si>
@@ -52,13 +59,16 @@
     <t>الاسم واللقب</t>
   </si>
   <si>
-    <t>08/09/2026</t>
+    <t>02/10/2026</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
     <t>بوكلوة ميار</t>
+  </si>
+  <si>
+    <t>بوناح سمر ميلينا</t>
   </si>
   <si>
     <t>تعليمات ملء الحضور والكتب / Instructions</t>
@@ -139,7 +149,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -176,6 +186,11 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F5FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -204,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -228,6 +243,9 @@
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -570,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -695,7 +713,7 @@
     </row>
     <row r="5" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
-        <v>550</v>
+        <v>389</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>9</v>
@@ -734,6 +752,50 @@
         <v>0</v>
       </c>
       <c r="N5" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>390</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="9">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9">
+        <v>0</v>
+      </c>
+      <c r="N6" s="9">
         <v>0</v>
       </c>
     </row>
@@ -760,8 +822,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>10</v>
+      <c r="A1" s="10" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -771,12 +833,12 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -786,27 +848,27 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -816,12 +878,12 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
@@ -831,7 +893,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>